<commit_message>
fix: unify F&B Production lab weights to BWCCI
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DwFtaYwDjsPSMtUxi63Qbw
</commit_message>
<xml_diff>
--- a/data/xlsx/isc-t-h--food-and-beverage-production-cooking.xlsx
+++ b/data/xlsx/isc-t-h--food-and-beverage-production-cooking.xlsx
@@ -722,7 +722,7 @@
         <v>0</v>
       </c>
       <c r="E19" s="9" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F19" s="9">
         <f>IFERROR(MIN(C19,D19)*E19/C19,0)</f>
@@ -914,7 +914,7 @@
         <v>0</v>
       </c>
       <c r="E27" s="9" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F27" s="9">
         <f>IFERROR(MIN(C27,D27)*E27/C27,0)</f>
@@ -938,7 +938,7 @@
         <v>0</v>
       </c>
       <c r="E28" s="9" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F28" s="9">
         <f>IFERROR(MIN(C28,D28)*E28/C28,0)</f>
@@ -962,7 +962,7 @@
         <v>0</v>
       </c>
       <c r="E29" s="9" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F29" s="9">
         <f>IFERROR(MIN(C29,D29)*E29/C29,0)</f>
@@ -1082,7 +1082,7 @@
         <v>0</v>
       </c>
       <c r="E34" s="9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F34" s="9">
         <f>IFERROR(MIN(C34,D34)*E34/C34,0)</f>

</xml_diff>